<commit_message>
feat: harden NVIDIA evidence and evaluation
</commit_message>
<xml_diff>
--- a/evaluation/week4/results/v2/week4_evaluation.xlsx
+++ b/evaluation/week4/results/v2/week4_evaluation.xlsx
@@ -675,10 +675,10 @@
         <v>3.344</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>3.728</v>
+        <v>4.058</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.384</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="15">
@@ -820,7 +820,7 @@
         <v>3.2857</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>3.7005</v>
+        <v>3.9652</v>
       </c>
     </row>
     <row r="3">
@@ -852,7 +852,7 @@
         <v>3.2323</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>3.5999</v>
+        <v>3.9869</v>
       </c>
     </row>
     <row r="4">
@@ -884,7 +884,7 @@
         <v>2.8822</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3.7275</v>
+        <v>3.9457</v>
       </c>
     </row>
     <row r="5">
@@ -916,7 +916,7 @@
         <v>3.1399</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>3.4269</v>
+        <v>3.8545</v>
       </c>
     </row>
     <row r="6">
@@ -948,7 +948,7 @@
         <v>2.7055</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>3.5481</v>
+        <v>3.9039</v>
       </c>
     </row>
     <row r="7">
@@ -980,7 +980,7 @@
         <v>3.1759</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>3.455</v>
+        <v>4.1688</v>
       </c>
     </row>
     <row r="8">
@@ -1012,7 +1012,7 @@
         <v>2.7242</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>3.6782</v>
+        <v>4.02</v>
       </c>
     </row>
     <row r="9">
@@ -1044,7 +1044,7 @@
         <v>3.0123</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3.454</v>
+        <v>3.8477</v>
       </c>
     </row>
     <row r="10">
@@ -1076,7 +1076,7 @@
         <v>3.0805</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>3.669</v>
+        <v>3.9222</v>
       </c>
     </row>
     <row r="11">
@@ -1108,7 +1108,7 @@
         <v>2.7534</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>3.4396</v>
+        <v>3.9138</v>
       </c>
     </row>
     <row r="12">
@@ -1140,7 +1140,7 @@
         <v>2.985</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>3.5955</v>
+        <v>3.8798</v>
       </c>
     </row>
     <row r="13">
@@ -1172,7 +1172,7 @@
         <v>4.0687</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>3.4483</v>
+        <v>3.8749</v>
       </c>
     </row>
     <row r="14">
@@ -1204,7 +1204,7 @@
         <v>3.2804</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>3.5398</v>
+        <v>3.8072</v>
       </c>
     </row>
     <row r="15">
@@ -1236,7 +1236,7 @@
         <v>3.1796</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>3.4844</v>
+        <v>3.9829</v>
       </c>
     </row>
     <row r="16">
@@ -1268,7 +1268,7 @@
         <v>3.0246</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>3.4465</v>
+        <v>3.7936</v>
       </c>
     </row>
     <row r="17">
@@ -1300,7 +1300,7 @@
         <v>3.2099</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>3.5753</v>
+        <v>3.9757</v>
       </c>
     </row>
     <row r="18">
@@ -1332,7 +1332,7 @@
         <v>3.1081</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>3.4745</v>
+        <v>3.8337</v>
       </c>
     </row>
     <row r="19">
@@ -1364,7 +1364,7 @@
         <v>3.3102</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>3.603</v>
+        <v>3.8681</v>
       </c>
     </row>
     <row r="20">
@@ -1396,7 +1396,7 @@
         <v>3.0491</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>3.655</v>
+        <v>3.9795</v>
       </c>
     </row>
     <row r="21">
@@ -1428,7 +1428,7 @@
         <v>2.6287</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>3.4812</v>
+        <v>3.9121</v>
       </c>
     </row>
     <row r="22">
@@ -1460,7 +1460,7 @@
         <v>3.2483</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>3.5432</v>
+        <v>4.0582</v>
       </c>
     </row>
     <row r="23">
@@ -1492,7 +1492,7 @@
         <v>3.1045</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>3.6142</v>
+        <v>3.9098</v>
       </c>
     </row>
     <row r="24">
@@ -1524,7 +1524,7 @@
         <v>3.2473</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>3.5599</v>
+        <v>4.0144</v>
       </c>
     </row>
     <row r="25">
@@ -1556,7 +1556,7 @@
         <v>3.3006</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>3.7787</v>
+        <v>4.0164</v>
       </c>
     </row>
     <row r="26">
@@ -1588,7 +1588,7 @@
         <v>3.0469</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>3.4261</v>
+        <v>3.8353</v>
       </c>
     </row>
     <row r="27">
@@ -1620,7 +1620,7 @@
         <v>3.1063</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>3.324</v>
+        <v>3.7298</v>
       </c>
     </row>
     <row r="28">
@@ -1652,7 +1652,7 @@
         <v>2.75</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>3.4661</v>
+        <v>3.7992</v>
       </c>
     </row>
     <row r="29">
@@ -1684,7 +1684,7 @@
         <v>2.8982</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>3.503</v>
+        <v>3.7982</v>
       </c>
     </row>
     <row r="30">
@@ -1716,7 +1716,7 @@
         <v>3.011</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>3.3511</v>
+        <v>3.7748</v>
       </c>
     </row>
     <row r="31">
@@ -1748,7 +1748,7 @@
         <v>3.119</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>3.3935</v>
+        <v>3.815</v>
       </c>
     </row>
     <row r="32">
@@ -1780,7 +1780,7 @@
         <v>2.9037</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>3.4363</v>
+        <v>3.9525</v>
       </c>
     </row>
     <row r="33">
@@ -1812,7 +1812,7 @@
         <v>2.9408</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>3.2065</v>
+        <v>3.7495</v>
       </c>
     </row>
     <row r="34">
@@ -1844,7 +1844,7 @@
         <v>2.8395</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>3.4532</v>
+        <v>3.7509</v>
       </c>
     </row>
     <row r="35">
@@ -1876,7 +1876,7 @@
         <v>3.3302</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>3.6002</v>
+        <v>4.1885</v>
       </c>
     </row>
     <row r="36">
@@ -1908,7 +1908,7 @@
         <v>3.1169</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>3.5772</v>
+        <v>3.8931</v>
       </c>
     </row>
     <row r="37">
@@ -1940,7 +1940,7 @@
         <v>3.3885</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>3.6934</v>
+        <v>3.963</v>
       </c>
     </row>
     <row r="38">
@@ -1972,7 +1972,7 @@
         <v>2.9548</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>3.5927</v>
+        <v>3.9097</v>
       </c>
     </row>
     <row r="39">
@@ -2004,7 +2004,7 @@
         <v>3.1277</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>3.4007</v>
+        <v>3.9203</v>
       </c>
     </row>
     <row r="40">
@@ -2036,7 +2036,7 @@
         <v>3.075</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>3.6302</v>
+        <v>3.8168</v>
       </c>
     </row>
     <row r="41">
@@ -2068,7 +2068,7 @@
         <v>3.0056</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>3.4443</v>
+        <v>3.7677</v>
       </c>
     </row>
     <row r="42">
@@ -2100,7 +2100,7 @@
         <v>3.2983</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>3.5451</v>
+        <v>3.9495</v>
       </c>
     </row>
     <row r="43">
@@ -2132,7 +2132,7 @@
         <v>3.1622</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>3.6355</v>
+        <v>3.841</v>
       </c>
     </row>
     <row r="44">
@@ -2164,7 +2164,7 @@
         <v>3.1165</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>3.403</v>
+        <v>3.8395</v>
       </c>
     </row>
     <row r="45">
@@ -2196,7 +2196,7 @@
         <v>2.8114</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>3.793</v>
+        <v>4.0026</v>
       </c>
     </row>
     <row r="46">
@@ -2228,7 +2228,7 @@
         <v>3.1902</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>3.877</v>
+        <v>3.9328</v>
       </c>
     </row>
     <row r="47">
@@ -2260,7 +2260,7 @@
         <v>3.6825</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>3.2512</v>
+        <v>3.8733</v>
       </c>
     </row>
     <row r="48">
@@ -2292,7 +2292,7 @@
         <v>3.1519</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>3.4929</v>
+        <v>3.7933</v>
       </c>
     </row>
     <row r="49">
@@ -2324,7 +2324,7 @@
         <v>2.8501</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>3.267</v>
+        <v>3.8863</v>
       </c>
     </row>
     <row r="50">
@@ -2356,7 +2356,7 @@
         <v>3.1911</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>3.6598</v>
+        <v>3.9053</v>
       </c>
     </row>
     <row r="51">
@@ -2388,7 +2388,7 @@
         <v>3.1909</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>3.5366</v>
+        <v>3.9108</v>
       </c>
     </row>
     <row r="52">
@@ -2420,7 +2420,7 @@
         <v>3.1277</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>3.4495</v>
+        <v>3.8971</v>
       </c>
     </row>
     <row r="53">
@@ -2452,7 +2452,7 @@
         <v>3.0921</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>3.4554</v>
+        <v>3.9221</v>
       </c>
     </row>
     <row r="54">
@@ -2484,7 +2484,7 @@
         <v>3.0139</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>3.4837</v>
+        <v>3.8372</v>
       </c>
     </row>
     <row r="55">
@@ -2516,7 +2516,7 @@
         <v>3.149</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>3.6415</v>
+        <v>3.9366</v>
       </c>
     </row>
     <row r="56">
@@ -2548,7 +2548,7 @@
         <v>3.1603</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>3.3233</v>
+        <v>3.9534</v>
       </c>
     </row>
     <row r="57">
@@ -2580,7 +2580,7 @@
         <v>3.0488</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>3.6697</v>
+        <v>3.9827</v>
       </c>
     </row>
     <row r="58">
@@ -2612,7 +2612,7 @@
         <v>3.9263</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>3.4172</v>
+        <v>3.8879</v>
       </c>
     </row>
     <row r="59">
@@ -2644,7 +2644,7 @@
         <v>2.9212</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>3.3047</v>
+        <v>3.9793</v>
       </c>
     </row>
     <row r="60">
@@ -2676,7 +2676,7 @@
         <v>3.0822</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>3.6047</v>
+        <v>3.928</v>
       </c>
     </row>
     <row r="61">
@@ -2708,7 +2708,7 @@
         <v>3.0306</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>3.5012</v>
+        <v>3.8884</v>
       </c>
     </row>
     <row r="62">
@@ -2740,7 +2740,7 @@
         <v>3.0622</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>3.6305</v>
+        <v>3.9486</v>
       </c>
     </row>
     <row r="63">
@@ -2772,7 +2772,7 @@
         <v>3.1364</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>3.5992</v>
+        <v>3.9281</v>
       </c>
     </row>
     <row r="64">
@@ -2804,7 +2804,7 @@
         <v>3.264</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>3.4721</v>
+        <v>3.9704</v>
       </c>
     </row>
     <row r="65">
@@ -2836,7 +2836,7 @@
         <v>3.1771</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>3.6711</v>
+        <v>3.9112</v>
       </c>
     </row>
     <row r="66">
@@ -2868,7 +2868,7 @@
         <v>3.1328</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>3.4978</v>
+        <v>3.9129</v>
       </c>
     </row>
     <row r="67">
@@ -2900,7 +2900,7 @@
         <v>3.1759</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>3.5842</v>
+        <v>4.0063</v>
       </c>
     </row>
     <row r="68">
@@ -2932,7 +2932,7 @@
         <v>2.8846</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>3.5844</v>
+        <v>3.9152</v>
       </c>
     </row>
     <row r="69">
@@ -2964,7 +2964,7 @@
         <v>3.2022</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>3.7334</v>
+        <v>3.9778</v>
       </c>
     </row>
     <row r="70">
@@ -2996,7 +2996,7 @@
         <v>3.3442</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>3.437</v>
+        <v>3.8957</v>
       </c>
     </row>
     <row r="71">
@@ -3028,7 +3028,7 @@
         <v>3.134</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>3.5238</v>
+        <v>3.9036</v>
       </c>
     </row>
     <row r="72">
@@ -3060,7 +3060,7 @@
         <v>3.3335</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>3.8788</v>
+        <v>3.9468</v>
       </c>
     </row>
     <row r="73">
@@ -3092,7 +3092,7 @@
         <v>3.3517</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>3.525</v>
+        <v>3.9747</v>
       </c>
     </row>
     <row r="74">
@@ -3124,7 +3124,7 @@
         <v>3.2583</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>3.517</v>
+        <v>3.8888</v>
       </c>
     </row>
     <row r="75">
@@ -3156,7 +3156,7 @@
         <v>3.0869</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>3.6527</v>
+        <v>3.9011</v>
       </c>
     </row>
     <row r="76">
@@ -3188,7 +3188,7 @@
         <v>3.224</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>3.5575</v>
+        <v>3.8942</v>
       </c>
     </row>
     <row r="77">
@@ -3220,7 +3220,7 @@
         <v>3.0043</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>3.2692</v>
+        <v>3.7591</v>
       </c>
     </row>
     <row r="78">
@@ -3252,7 +3252,7 @@
         <v>3.0719</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>3.4543</v>
+        <v>3.976</v>
       </c>
     </row>
     <row r="79">
@@ -3284,7 +3284,7 @@
         <v>3.1896</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>3.6901</v>
+        <v>3.9865</v>
       </c>
     </row>
     <row r="80">
@@ -3316,7 +3316,7 @@
         <v>3.0006</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>3.3881</v>
+        <v>3.8216</v>
       </c>
     </row>
     <row r="81">
@@ -3348,7 +3348,7 @@
         <v>3.0588</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>3.1508</v>
+        <v>3.7981</v>
       </c>
     </row>
     <row r="82">
@@ -3380,7 +3380,7 @@
         <v>3.0695</v>
       </c>
       <c r="H82" s="3" t="n">
-        <v>3.3574</v>
+        <v>3.7767</v>
       </c>
     </row>
     <row r="83">
@@ -3412,7 +3412,7 @@
         <v>2.8749</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>3.5706</v>
+        <v>3.7528</v>
       </c>
     </row>
     <row r="84">
@@ -3444,7 +3444,7 @@
         <v>3.031</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>3.4397</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="85">
@@ -3476,7 +3476,7 @@
         <v>3.3167</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>3.5302</v>
+        <v>3.9065</v>
       </c>
     </row>
     <row r="86">
@@ -3508,7 +3508,7 @@
         <v>3.1592</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>3.6369</v>
+        <v>3.9365</v>
       </c>
     </row>
     <row r="87">
@@ -3540,7 +3540,7 @@
         <v>3.113</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>3.4169</v>
+        <v>4.0177</v>
       </c>
     </row>
     <row r="88">
@@ -3572,7 +3572,7 @@
         <v>2.6691</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>3.5415</v>
+        <v>3.9096</v>
       </c>
     </row>
     <row r="89">
@@ -3604,7 +3604,7 @@
         <v>3.0282</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>3.6233</v>
+        <v>3.8848</v>
       </c>
     </row>
     <row r="90">
@@ -3636,7 +3636,7 @@
         <v>3.1419</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>3.6913</v>
+        <v>4.1852</v>
       </c>
     </row>
     <row r="91">
@@ -3668,7 +3668,7 @@
         <v>2.7924</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>3.5628</v>
+        <v>4.009</v>
       </c>
     </row>
     <row r="92">
@@ -3700,7 +3700,7 @@
         <v>3.2169</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>3.3714</v>
+        <v>4.0761</v>
       </c>
     </row>
     <row r="93">
@@ -3732,7 +3732,7 @@
         <v>2.8126</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>3.5183</v>
+        <v>3.8905</v>
       </c>
     </row>
     <row r="94">
@@ -3764,7 +3764,7 @@
         <v>2.9813</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>3.4334</v>
+        <v>3.8972</v>
       </c>
     </row>
     <row r="95">
@@ -3796,7 +3796,7 @@
         <v>3.0788</v>
       </c>
       <c r="H95" s="3" t="n">
-        <v>3.5209</v>
+        <v>3.8942</v>
       </c>
     </row>
     <row r="96">
@@ -3828,7 +3828,7 @@
         <v>2.795</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>3.5306</v>
+        <v>3.8792</v>
       </c>
     </row>
     <row r="97">
@@ -3860,7 +3860,7 @@
         <v>3.145</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>3.5374</v>
+        <v>3.9135</v>
       </c>
     </row>
     <row r="98">
@@ -3892,7 +3892,7 @@
         <v>3.0483</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>3.4125</v>
+        <v>4.0921</v>
       </c>
     </row>
     <row r="99">
@@ -3924,7 +3924,7 @@
         <v>2.7233</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>3.344</v>
+        <v>3.9054</v>
       </c>
     </row>
     <row r="100">
@@ -3956,7 +3956,7 @@
         <v>2.7503</v>
       </c>
       <c r="H100" s="3" t="n">
-        <v>3.6111</v>
+        <v>3.853</v>
       </c>
     </row>
     <row r="101">
@@ -3988,7 +3988,7 @@
         <v>2.8919</v>
       </c>
       <c r="H101" s="3" t="n">
-        <v>3.64</v>
+        <v>3.7704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>